<commit_message>
Deploying to gh-pages from @ HiLiftPW-Committee/HiLiftPW-Committee.github.io@76f32a4367b7c24143ef3d550a9b7a50159431a3 🚀
</commit_message>
<xml_diff>
--- a/assets/HLPW6/tc1/TC1_Pressure_Rows.xlsx
+++ b/assets/HLPW6/tc1/TC1_Pressure_Rows.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\nos\Data\CRMHL_EC\External Communication\HLPW6\Test_Cases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\heathcote.daniel\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F186AF5A-6376-4F88-ABBE-7C9576337F1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D1467A4-DCA1-426B-8BBA-AC7845A1CDB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23172" yWindow="8976" windowWidth="23304" windowHeight="12504" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="41">
   <si>
     <t>Belt</t>
   </si>
@@ -156,6 +156,9 @@
   </si>
   <si>
     <t>Flap</t>
+  </si>
+  <si>
+    <t>Plane orientation equation coefficients</t>
   </si>
 </sst>
 </file>
@@ -250,25 +253,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -293,14 +294,14 @@
     <xdr:from>
       <xdr:col>12</xdr:col>
       <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>0</xdr:row>
+      <xdr:row>1</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>11207</xdr:rowOff>
+      <xdr:colOff>121285</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>8667</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -343,13 +344,13 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>552450</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>40</xdr:row>
+      <xdr:row>41</xdr:row>
       <xdr:rowOff>77123</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -655,90 +656,61 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A2:R35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.85546875" customWidth="1"/>
+    <col min="1" max="1" width="4.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="H1" s="3" t="s">
+      <c r="B2" s="2"/>
+      <c r="C2" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="H2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="3"/>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="I2" s="3"/>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="B3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2" t="s">
+      <c r="G3" s="2"/>
+      <c r="H3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J3" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B4" s="5" t="s">
         <v>5</v>
-      </c>
-      <c r="C3">
-        <v>6.4508999999999997E-2</v>
-      </c>
-      <c r="D3">
-        <v>0.95106599999999997</v>
-      </c>
-      <c r="E3">
-        <v>-0.302178</v>
-      </c>
-      <c r="F3">
-        <v>12.0589</v>
-      </c>
-      <c r="H3" s="1">
-        <v>9.9523520600000008</v>
-      </c>
-      <c r="I3" s="1">
-        <v>12.02716081</v>
-      </c>
-      <c r="J3" s="1">
-        <v>7.2001480000000007E-2</v>
-      </c>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
-      <c r="P3" s="1"/>
-      <c r="Q3" s="1"/>
-      <c r="R3" s="1"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" s="13"/>
-      <c r="B4" s="9" t="s">
-        <v>6</v>
       </c>
       <c r="C4">
         <v>6.4508999999999997E-2</v>
@@ -749,29 +721,31 @@
       <c r="E4">
         <v>-0.302178</v>
       </c>
-      <c r="F4" s="5">
-        <v>18.9069</v>
+      <c r="F4">
+        <v>12.0589</v>
       </c>
       <c r="H4" s="1">
-        <v>15.14698035</v>
-      </c>
-      <c r="I4">
-        <v>18.8751608</v>
+        <v>9.9523520600000008</v>
+      </c>
+      <c r="I4" s="1">
+        <v>12.02716081</v>
       </c>
       <c r="J4" s="1">
         <v>7.2001480000000007E-2</v>
       </c>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
       <c r="P4" s="1"/>
+      <c r="Q4" s="1"/>
       <c r="R4" s="1"/>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A5" s="13"/>
-      <c r="B5" s="9" t="s">
-        <v>7</v>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A5" s="9"/>
+      <c r="B5" s="5" t="s">
+        <v>6</v>
       </c>
       <c r="C5">
         <v>6.4508999999999997E-2</v>
@@ -782,31 +756,29 @@
       <c r="E5">
         <v>-0.302178</v>
       </c>
-      <c r="F5" s="5">
-        <v>35.058900000000001</v>
+      <c r="F5">
+        <v>18.9069</v>
       </c>
       <c r="H5" s="1">
-        <v>27.399263680000001</v>
-      </c>
-      <c r="I5" s="1">
-        <v>35.027160790000003</v>
+        <v>15.14698035</v>
+      </c>
+      <c r="I5">
+        <v>18.8751608</v>
       </c>
       <c r="J5" s="1">
         <v>7.2001480000000007E-2</v>
       </c>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
-      <c r="Q5" s="1"/>
       <c r="R5" s="1"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A6" s="13"/>
-      <c r="B6" s="9" t="s">
-        <v>8</v>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A6" s="9"/>
+      <c r="B6" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="C6">
         <v>6.4508999999999997E-2</v>
@@ -817,14 +789,14 @@
       <c r="E6">
         <v>-0.302178</v>
       </c>
-      <c r="F6" s="5">
-        <v>47.058900000000001</v>
+      <c r="F6">
+        <v>35.058900000000001</v>
       </c>
       <c r="H6" s="1">
-        <v>36.502000170000002</v>
+        <v>27.399263680000001</v>
       </c>
       <c r="I6" s="1">
-        <v>47.027160790000003</v>
+        <v>35.027160790000003</v>
       </c>
       <c r="J6" s="1">
         <v>7.2001480000000007E-2</v>
@@ -838,10 +810,10 @@
       <c r="Q6" s="1"/>
       <c r="R6" s="1"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A7" s="13"/>
-      <c r="B7" s="9" t="s">
-        <v>9</v>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A7" s="9"/>
+      <c r="B7" s="5" t="s">
+        <v>8</v>
       </c>
       <c r="C7">
         <v>6.4508999999999997E-2</v>
@@ -852,14 +824,14 @@
       <c r="E7">
         <v>-0.302178</v>
       </c>
-      <c r="F7" s="5">
-        <v>52.962899999999998</v>
+      <c r="F7">
+        <v>47.058900000000001</v>
       </c>
       <c r="H7" s="1">
-        <v>40.980546529999998</v>
+        <v>36.502000170000002</v>
       </c>
       <c r="I7" s="1">
-        <v>52.931160779999999</v>
+        <v>47.027160790000003</v>
       </c>
       <c r="J7" s="1">
         <v>7.2001480000000007E-2</v>
@@ -873,10 +845,10 @@
       <c r="Q7" s="1"/>
       <c r="R7" s="1"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A8" s="13"/>
-      <c r="B8" s="9" t="s">
-        <v>10</v>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A8" s="9"/>
+      <c r="B8" s="5" t="s">
+        <v>9</v>
       </c>
       <c r="C8">
         <v>6.4508999999999997E-2</v>
@@ -887,14 +859,14 @@
       <c r="E8">
         <v>-0.302178</v>
       </c>
-      <c r="F8" s="5">
-        <v>59.058900000000001</v>
+      <c r="F8">
+        <v>52.962899999999998</v>
       </c>
       <c r="H8" s="1">
-        <v>45.604736670000001</v>
+        <v>40.980546529999998</v>
       </c>
       <c r="I8" s="1">
-        <v>59.027160780000003</v>
+        <v>52.931160779999999</v>
       </c>
       <c r="J8" s="1">
         <v>7.2001480000000007E-2</v>
@@ -908,10 +880,10 @@
       <c r="Q8" s="1"/>
       <c r="R8" s="1"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A9" s="13"/>
-      <c r="B9" s="9" t="s">
-        <v>33</v>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A9" s="9"/>
+      <c r="B9" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="C9">
         <v>6.4508999999999997E-2</v>
@@ -922,14 +894,14 @@
       <c r="E9">
         <v>-0.302178</v>
       </c>
-      <c r="F9" s="5">
-        <v>70.058899999999994</v>
+      <c r="F9">
+        <v>59.058900000000001</v>
       </c>
       <c r="H9" s="1">
-        <v>53.948911789999997</v>
+        <v>45.604736670000001</v>
       </c>
       <c r="I9" s="1">
-        <v>70.027160769999995</v>
+        <v>59.027160780000003</v>
       </c>
       <c r="J9" s="1">
         <v>7.2001480000000007E-2</v>
@@ -943,16 +915,32 @@
       <c r="Q9" s="1"/>
       <c r="R9" s="1"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A10" s="14"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A10" s="9"/>
+      <c r="B10" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10">
+        <v>6.4508999999999997E-2</v>
+      </c>
+      <c r="D10">
+        <v>0.95106599999999997</v>
+      </c>
+      <c r="E10">
+        <v>-0.302178</v>
+      </c>
+      <c r="F10">
+        <v>70.058899999999994</v>
+      </c>
+      <c r="H10" s="1">
+        <v>53.948911789999997</v>
+      </c>
+      <c r="I10" s="1">
+        <v>70.027160769999995</v>
+      </c>
+      <c r="J10" s="1">
+        <v>7.2001480000000007E-2</v>
+      </c>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
@@ -962,62 +950,45 @@
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A11" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="5">
-        <v>0</v>
-      </c>
-      <c r="D11" s="5">
-        <v>1</v>
-      </c>
-      <c r="E11" s="5">
-        <v>0</v>
-      </c>
-      <c r="F11" s="5">
-        <v>10</v>
-      </c>
-      <c r="H11" s="1">
-        <v>33.460999999999999</v>
-      </c>
-      <c r="I11" s="1">
-        <v>10</v>
-      </c>
-      <c r="J11" s="1">
-        <v>0.85</v>
-      </c>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A11" s="8"/>
+      <c r="B11" s="3"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
       <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
       <c r="O11" s="1"/>
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
       <c r="R11" s="1"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A12" s="13"/>
-      <c r="B12" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" s="5">
-        <v>0</v>
-      </c>
-      <c r="D12" s="5">
-        <v>1</v>
-      </c>
-      <c r="E12" s="5">
-        <v>0</v>
-      </c>
-      <c r="F12" s="5">
-        <v>16.847999999999999</v>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>10</v>
       </c>
       <c r="H12" s="1">
-        <v>38.655000000000001</v>
-      </c>
-      <c r="I12">
-        <v>16.847999999999999</v>
+        <v>33.460999999999999</v>
+      </c>
+      <c r="I12" s="1">
+        <v>10</v>
       </c>
       <c r="J12" s="1">
         <v>0.85</v>
@@ -1025,30 +996,31 @@
       <c r="K12" s="1"/>
       <c r="O12" s="1"/>
       <c r="P12" s="1"/>
+      <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A13" s="13"/>
-      <c r="B13" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" s="5">
-        <v>0</v>
-      </c>
-      <c r="D13" s="5">
-        <v>1</v>
-      </c>
-      <c r="E13" s="5">
-        <v>0</v>
-      </c>
-      <c r="F13" s="5">
-        <v>33</v>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A13" s="9"/>
+      <c r="B13" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>16.847999999999999</v>
       </c>
       <c r="H13" s="1">
-        <v>50.908000000000001</v>
-      </c>
-      <c r="I13" s="1">
-        <v>33</v>
+        <v>38.655000000000001</v>
+      </c>
+      <c r="I13">
+        <v>16.847999999999999</v>
       </c>
       <c r="J13" s="1">
         <v>0.85</v>
@@ -1056,34 +1028,33 @@
       <c r="K13" s="1"/>
       <c r="O13" s="1"/>
       <c r="P13" s="1"/>
-      <c r="Q13" s="1"/>
       <c r="R13" s="1"/>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A14" s="13"/>
-      <c r="B14" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="5">
-        <v>0</v>
-      </c>
-      <c r="D14" s="5">
-        <v>1</v>
-      </c>
-      <c r="E14" s="5">
-        <v>0</v>
-      </c>
-      <c r="F14" s="5">
-        <v>45</v>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A14" s="9"/>
+      <c r="B14" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>33</v>
       </c>
       <c r="H14" s="1">
-        <v>64.135999999999996</v>
+        <v>50.908000000000001</v>
       </c>
       <c r="I14" s="1">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="J14" s="1">
-        <v>1.7999999999999999E-2</v>
+        <v>0.85</v>
       </c>
       <c r="K14" s="1"/>
       <c r="O14" s="1"/>
@@ -1091,31 +1062,31 @@
       <c r="Q14" s="1"/>
       <c r="R14" s="1"/>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A15" s="13"/>
-      <c r="B15" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" s="5">
-        <v>0</v>
-      </c>
-      <c r="D15" s="5">
-        <v>1</v>
-      </c>
-      <c r="E15" s="5">
-        <v>0</v>
-      </c>
-      <c r="F15" s="5">
-        <v>50.904000000000003</v>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A15" s="9"/>
+      <c r="B15" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>45</v>
       </c>
       <c r="H15" s="1">
-        <v>68.614000000000004</v>
+        <v>64.135999999999996</v>
       </c>
       <c r="I15" s="1">
-        <v>50.904000000000003</v>
+        <v>45</v>
       </c>
       <c r="J15" s="1">
-        <v>0.85</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="K15" s="1"/>
       <c r="O15" s="1"/>
@@ -1123,28 +1094,28 @@
       <c r="Q15" s="1"/>
       <c r="R15" s="1"/>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A16" s="13"/>
-      <c r="B16" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C16" s="5">
-        <v>0</v>
-      </c>
-      <c r="D16" s="5">
-        <v>1</v>
-      </c>
-      <c r="E16" s="5">
-        <v>0</v>
-      </c>
-      <c r="F16" s="5">
-        <v>57</v>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A16" s="9"/>
+      <c r="B16" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16">
+        <v>0</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>50.904000000000003</v>
       </c>
       <c r="H16" s="1">
-        <v>81.582999999999998</v>
+        <v>68.614000000000004</v>
       </c>
       <c r="I16" s="1">
-        <v>68</v>
+        <v>50.904000000000003</v>
       </c>
       <c r="J16" s="1">
         <v>0.85</v>
@@ -1155,28 +1126,28 @@
       <c r="Q16" s="1"/>
       <c r="R16" s="1"/>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A17" s="13"/>
-      <c r="B17" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C17" s="5">
-        <v>0</v>
-      </c>
-      <c r="D17" s="5">
-        <v>1</v>
-      </c>
-      <c r="E17" s="5">
-        <v>0</v>
-      </c>
-      <c r="F17" s="5">
-        <v>68</v>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A17" s="9"/>
+      <c r="B17" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17">
+        <v>0</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>57</v>
       </c>
       <c r="H17" s="1">
         <v>81.582999999999998</v>
       </c>
       <c r="I17" s="1">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="J17" s="1">
         <v>0.85</v>
@@ -1187,81 +1158,77 @@
       <c r="Q17" s="1"/>
       <c r="R17" s="1"/>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A18" s="14"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A18" s="9"/>
+      <c r="B18" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>68</v>
+      </c>
+      <c r="H18" s="1">
+        <v>81.582999999999998</v>
+      </c>
+      <c r="I18" s="1">
+        <v>68</v>
+      </c>
+      <c r="J18" s="1">
+        <v>0.85</v>
+      </c>
       <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
       <c r="O18" s="1"/>
       <c r="P18" s="1"/>
       <c r="Q18" s="1"/>
       <c r="R18" s="1"/>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A19" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C19" s="5">
-        <v>0</v>
-      </c>
-      <c r="D19" s="5">
-        <v>1</v>
-      </c>
-      <c r="E19" s="5">
-        <v>0</v>
-      </c>
-      <c r="F19" s="5">
-        <v>10</v>
-      </c>
-      <c r="H19" s="1">
-        <v>38.854999999999997</v>
-      </c>
-      <c r="I19" s="1">
-        <v>10</v>
-      </c>
-      <c r="J19" s="1">
-        <v>-3.6</v>
-      </c>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A19" s="8"/>
+      <c r="B19" s="3"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
       <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
       <c r="O19" s="1"/>
       <c r="P19" s="1"/>
       <c r="Q19" s="1"/>
       <c r="R19" s="1"/>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A20" s="13"/>
-      <c r="B20" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C20" s="5">
-        <v>0</v>
-      </c>
-      <c r="D20" s="5">
-        <v>1</v>
-      </c>
-      <c r="E20" s="5">
-        <v>0</v>
-      </c>
-      <c r="F20" s="5">
-        <v>16.847999999999999</v>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A20" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>10</v>
       </c>
       <c r="H20" s="1">
-        <v>44.05</v>
-      </c>
-      <c r="I20">
-        <v>16.847999999999999</v>
+        <v>38.854999999999997</v>
+      </c>
+      <c r="I20" s="1">
+        <v>10</v>
       </c>
       <c r="J20" s="1">
         <v>-3.6</v>
@@ -1269,12 +1236,13 @@
       <c r="K20" s="1"/>
       <c r="O20" s="1"/>
       <c r="P20" s="1"/>
+      <c r="Q20" s="1"/>
       <c r="R20" s="1"/>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A21" s="13"/>
-      <c r="B21" s="12" t="s">
-        <v>21</v>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A21" s="9"/>
+      <c r="B21" s="7" t="s">
+        <v>20</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -1286,13 +1254,13 @@
         <v>0</v>
       </c>
       <c r="F21">
-        <v>33</v>
+        <v>16.847999999999999</v>
       </c>
       <c r="H21" s="1">
-        <v>56.301000000000002</v>
-      </c>
-      <c r="I21" s="1">
-        <v>33</v>
+        <v>44.05</v>
+      </c>
+      <c r="I21">
+        <v>16.847999999999999</v>
       </c>
       <c r="J21" s="1">
         <v>-3.6</v>
@@ -1300,330 +1268,326 @@
       <c r="K21" s="1"/>
       <c r="O21" s="1"/>
       <c r="P21" s="1"/>
-      <c r="Q21" s="1"/>
       <c r="R21" s="1"/>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A22" s="14"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="J22" s="1"/>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A22" s="9"/>
+      <c r="B22" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22">
+        <v>33</v>
+      </c>
+      <c r="H22" s="1">
+        <v>56.301000000000002</v>
+      </c>
+      <c r="I22" s="1">
+        <v>33</v>
+      </c>
+      <c r="J22" s="1">
+        <v>-3.6</v>
+      </c>
       <c r="K22" s="1"/>
-      <c r="L22" s="1"/>
-      <c r="M22" s="1"/>
-      <c r="N22" s="1"/>
       <c r="O22" s="1"/>
       <c r="P22" s="1"/>
       <c r="Q22" s="1"/>
       <c r="R22" s="1"/>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A23" s="14"/>
-      <c r="B23" s="2" t="s">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A23" s="8"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="P23" s="1"/>
+      <c r="Q23" s="1"/>
+      <c r="R23" s="1"/>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A24" s="8"/>
+      <c r="B24" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A24" s="14"/>
-      <c r="B24" s="2"/>
-      <c r="D24" t="s">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A25" s="8"/>
+      <c r="B25" s="2"/>
+      <c r="D25" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A25" s="14"/>
-      <c r="B25" s="2"/>
-      <c r="H25" s="3" t="s">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A26" s="8"/>
+      <c r="B26" s="2"/>
+      <c r="H26" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="I25" s="3"/>
-      <c r="J25" s="3"/>
-    </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A26" s="14"/>
-      <c r="B26" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="D26" s="6" t="s">
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A27" s="8"/>
+      <c r="B27" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="E27" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F26" s="6" t="s">
+      <c r="F27" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G26" s="7"/>
-      <c r="H26" s="6" t="s">
+      <c r="G27" s="4"/>
+      <c r="H27" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="I26" s="6" t="s">
+      <c r="I27" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="J26" s="6" t="s">
+      <c r="J27" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="K26" s="5"/>
-    </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A27" s="13" t="s">
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A28" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B28" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C27" s="5">
+      <c r="C28">
         <v>0.79671499999999995</v>
       </c>
-      <c r="D27" s="5">
+      <c r="D28">
         <v>-0.604356</v>
       </c>
-      <c r="E27" s="5">
-        <v>0</v>
-      </c>
-      <c r="F27" s="5">
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
         <v>3.4660000000000002</v>
       </c>
-      <c r="G27" s="5"/>
-      <c r="H27" s="5">
+      <c r="H28">
         <v>5.1085600199999996</v>
       </c>
-      <c r="I27" s="5">
-        <v>1</v>
-      </c>
-      <c r="J27" s="5">
+      <c r="I28">
+        <v>1</v>
+      </c>
+      <c r="J28">
         <v>1.1549626799999999</v>
       </c>
-      <c r="K27" s="5"/>
-      <c r="L27" s="1"/>
-      <c r="M27" s="1"/>
-      <c r="N27" s="1"/>
-    </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A28" s="13"/>
-      <c r="B28" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C28" s="5">
-        <v>0.79671499999999995</v>
-      </c>
-      <c r="D28" s="5">
-        <v>-0.604356</v>
-      </c>
-      <c r="E28" s="5">
-        <v>0</v>
-      </c>
-      <c r="F28" s="5">
-        <v>6.931</v>
-      </c>
-      <c r="G28" s="5"/>
-      <c r="H28" s="5">
-        <v>9.4585600200000002</v>
-      </c>
-      <c r="I28" s="5">
-        <v>1</v>
-      </c>
-      <c r="J28" s="5">
-        <v>1.5428141799999999</v>
-      </c>
-      <c r="K28" s="5"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
       <c r="N28" s="1"/>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A29" s="13"/>
-      <c r="B29" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C29" s="5">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A29" s="9"/>
+      <c r="B29" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C29">
         <v>0.79671499999999995</v>
       </c>
-      <c r="D29" s="5">
+      <c r="D29">
         <v>-0.604356</v>
       </c>
-      <c r="E29" s="5">
-        <v>0</v>
-      </c>
-      <c r="F29" s="5">
-        <v>10.397</v>
-      </c>
-      <c r="G29" s="5"/>
-      <c r="H29" s="5">
-        <v>13.80856002</v>
-      </c>
-      <c r="I29" s="5">
-        <v>1</v>
-      </c>
-      <c r="J29" s="5">
-        <v>1.6527511699999999</v>
-      </c>
-      <c r="K29" s="5"/>
+      <c r="E29">
+        <v>0</v>
+      </c>
+      <c r="F29">
+        <v>6.931</v>
+      </c>
+      <c r="H29">
+        <v>9.4585600200000002</v>
+      </c>
+      <c r="I29">
+        <v>1</v>
+      </c>
+      <c r="J29">
+        <v>1.5428141799999999</v>
+      </c>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
       <c r="N29" s="1"/>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A30" s="13"/>
-      <c r="B30" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C30" s="5">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A30" s="9"/>
+      <c r="B30" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C30">
         <v>0.79671499999999995</v>
       </c>
-      <c r="D30" s="5">
+      <c r="D30">
         <v>-0.604356</v>
       </c>
-      <c r="E30" s="5">
-        <v>0</v>
-      </c>
-      <c r="F30" s="5">
-        <v>13.911</v>
-      </c>
-      <c r="G30" s="5"/>
-      <c r="H30" s="5">
-        <v>18.218560020000002</v>
-      </c>
-      <c r="I30" s="5">
-        <v>1</v>
-      </c>
-      <c r="J30" s="5">
-        <v>1.5960287099999999</v>
-      </c>
-      <c r="K30" s="5"/>
+      <c r="E30">
+        <v>0</v>
+      </c>
+      <c r="F30">
+        <v>10.397</v>
+      </c>
+      <c r="H30">
+        <v>13.80856002</v>
+      </c>
+      <c r="I30">
+        <v>1</v>
+      </c>
+      <c r="J30">
+        <v>1.6527511699999999</v>
+      </c>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
       <c r="N30" s="1"/>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A31" s="13"/>
-      <c r="B31" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C31" s="5">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A31" s="9"/>
+      <c r="B31" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C31">
         <v>0.79671499999999995</v>
       </c>
-      <c r="D31" s="5">
+      <c r="D31">
         <v>-0.604356</v>
       </c>
-      <c r="E31" s="5">
-        <v>0</v>
-      </c>
-      <c r="F31" s="5">
-        <v>17.352</v>
-      </c>
-      <c r="G31" s="5"/>
-      <c r="H31" s="5">
-        <v>22.538560019999998</v>
-      </c>
-      <c r="I31" s="5">
-        <v>1</v>
-      </c>
-      <c r="J31" s="5">
-        <v>1.33398678</v>
-      </c>
-      <c r="K31" s="5"/>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <v>13.911</v>
+      </c>
+      <c r="H31">
+        <v>18.218560020000002</v>
+      </c>
+      <c r="I31">
+        <v>1</v>
+      </c>
+      <c r="J31">
+        <v>1.5960287099999999</v>
+      </c>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
       <c r="N31" s="1"/>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A32" s="13"/>
-      <c r="B32" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C32" s="5">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A32" s="9"/>
+      <c r="B32" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C32">
         <v>0.79671499999999995</v>
       </c>
-      <c r="D32" s="5">
+      <c r="D32">
         <v>-0.604356</v>
       </c>
-      <c r="E32" s="5">
-        <v>0</v>
-      </c>
-      <c r="F32" s="5">
-        <v>21.105</v>
-      </c>
-      <c r="G32" s="5"/>
-      <c r="H32" s="5">
-        <v>53.798160680000002</v>
-      </c>
-      <c r="I32" s="5">
-        <v>36</v>
-      </c>
-      <c r="J32" s="5">
-        <v>0.76525666000000003</v>
-      </c>
-      <c r="K32" s="5"/>
+      <c r="E32">
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <v>17.352</v>
+      </c>
+      <c r="H32">
+        <v>22.538560019999998</v>
+      </c>
+      <c r="I32">
+        <v>1</v>
+      </c>
+      <c r="J32">
+        <v>1.33398678</v>
+      </c>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
       <c r="N32" s="1"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" s="14"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="5"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
-      <c r="G33" s="5"/>
-      <c r="H33" s="5"/>
-      <c r="I33" s="5"/>
-      <c r="J33" s="5"/>
-      <c r="K33" s="5"/>
-    </row>
-    <row r="34" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A34" s="14" t="s">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A33" s="9"/>
+      <c r="B33" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C33">
+        <v>0.79671499999999995</v>
+      </c>
+      <c r="D33">
+        <v>-0.604356</v>
+      </c>
+      <c r="E33">
+        <v>0</v>
+      </c>
+      <c r="F33">
+        <v>21.105</v>
+      </c>
+      <c r="H33">
+        <v>53.798160680000002</v>
+      </c>
+      <c r="I33">
+        <v>36</v>
+      </c>
+      <c r="J33">
+        <v>0.76525666000000003</v>
+      </c>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A34" s="8"/>
+      <c r="B34" s="3"/>
+    </row>
+    <row r="35" spans="1:14" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A35" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B35" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C34" s="5">
+      <c r="C35">
         <v>0.79671499999999995</v>
       </c>
-      <c r="D34" s="5">
+      <c r="D35">
         <v>-0.604356</v>
       </c>
-      <c r="E34" s="5">
-        <v>0</v>
-      </c>
-      <c r="F34" s="5">
+      <c r="E35">
+        <v>0</v>
+      </c>
+      <c r="F35">
         <v>21.105</v>
       </c>
-      <c r="G34" s="5"/>
-      <c r="H34" s="5">
+      <c r="H35">
         <v>29.278631820000001</v>
       </c>
-      <c r="I34" s="5">
+      <c r="I35">
         <v>3.6762177700000001</v>
       </c>
-      <c r="J34" s="5">
+      <c r="J35">
         <v>0.50722509000000005</v>
       </c>
-      <c r="K34" s="5"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B35" s="5"/>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
-      <c r="H35" s="5"/>
-      <c r="I35" s="5"/>
-      <c r="J35" s="5"/>
-      <c r="K35" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A3:A9"/>
-    <mergeCell ref="A11:A17"/>
-    <mergeCell ref="A27:A32"/>
-    <mergeCell ref="A19:A21"/>
+  <mergeCells count="5">
+    <mergeCell ref="A4:A10"/>
+    <mergeCell ref="A12:A18"/>
+    <mergeCell ref="A28:A33"/>
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="C2:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>